<commit_message>
Zapis do wynikow do 3 arkuszy excela
</commit_message>
<xml_diff>
--- a/Backend/config/uploaded_template.xlsx
+++ b/Backend/config/uploaded_template.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="163" documentId="11_33AB73D7375CF2584D5B4BDD7E1B1DA65E074F86" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E13063B-321F-4798-88D7-45B69B19ED6E}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1" sheetId="74" r:id="rId1"/>
@@ -7179,24 +7179,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:GA76"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="10.199999999999999" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4" style="9" customWidth="1"/>
-    <col min="2" max="2" width="3.42578125" style="9" customWidth="1"/>
+    <col min="2" max="2" width="3.44140625" style="9" customWidth="1"/>
     <col min="3" max="3" width="7" style="8" customWidth="1"/>
-    <col min="4" max="4" width="1.42578125" style="8" customWidth="1"/>
+    <col min="4" max="4" width="1.44140625" style="8" customWidth="1"/>
     <col min="5" max="8" width="9" style="8" customWidth="1"/>
-    <col min="9" max="16" width="5.5703125" style="8" customWidth="1"/>
+    <col min="9" max="16" width="5.5546875" style="8" customWidth="1"/>
     <col min="17" max="17" width="3" style="2" customWidth="1"/>
-    <col min="18" max="18" width="4.140625" style="2" customWidth="1"/>
+    <col min="18" max="18" width="4.109375" style="2" customWidth="1"/>
     <col min="19" max="19" width="3" style="2" customWidth="1"/>
-    <col min="20" max="29" width="10.85546875" style="2" customWidth="1"/>
-    <col min="30" max="30" width="11.42578125" style="11"/>
-    <col min="31" max="35" width="11.42578125" style="7"/>
-    <col min="36" max="16384" width="11.42578125" style="8"/>
+    <col min="20" max="29" width="10.88671875" style="2" customWidth="1"/>
+    <col min="30" max="30" width="11.44140625" style="11"/>
+    <col min="31" max="35" width="11.44140625" style="7"/>
+    <col min="36" max="16384" width="11.44140625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:183" s="4" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:183" s="4" customFormat="1" ht="10.8" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="78"/>
       <c r="B1" s="78"/>
       <c r="C1" s="78"/>
@@ -7384,7 +7384,7 @@
       <c r="AH4" s="3"/>
       <c r="AI4" s="3"/>
     </row>
-    <row r="5" spans="1:183" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:183" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="78"/>
       <c r="B5" s="102" t="s">
         <v>4</v>
@@ -7427,7 +7427,7 @@
       <c r="AH5" s="3"/>
       <c r="AI5" s="3"/>
     </row>
-    <row r="6" spans="1:183" s="5" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:183" s="5" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="72"/>
       <c r="B6" s="106"/>
       <c r="C6" s="72"/>
@@ -7933,7 +7933,7 @@
       <c r="AF12" s="3"/>
       <c r="AG12" s="3"/>
     </row>
-    <row r="13" spans="1:183" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:183" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="82"/>
       <c r="B13" s="78"/>
       <c r="C13" s="268" t="s">
@@ -10319,30 +10319,30 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:GA76"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="10.199999999999999" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4" style="9" customWidth="1"/>
-    <col min="2" max="2" width="3.42578125" style="9" customWidth="1"/>
+    <col min="2" max="2" width="3.44140625" style="9" customWidth="1"/>
     <col min="3" max="3" width="7" style="8" customWidth="1"/>
-    <col min="4" max="4" width="1.42578125" style="8" customWidth="1"/>
+    <col min="4" max="4" width="1.44140625" style="8" customWidth="1"/>
     <col min="5" max="8" width="9" style="8" customWidth="1"/>
-    <col min="9" max="11" width="5.5703125" style="8" customWidth="1"/>
-    <col min="12" max="12" width="11.85546875" style="8" customWidth="1"/>
-    <col min="13" max="13" width="5.5703125" style="8" customWidth="1"/>
-    <col min="14" max="14" width="8.7109375" style="8" customWidth="1"/>
-    <col min="15" max="15" width="5.5703125" style="8" customWidth="1"/>
-    <col min="16" max="16" width="13.5703125" style="8" customWidth="1"/>
+    <col min="9" max="11" width="5.5546875" style="8" customWidth="1"/>
+    <col min="12" max="12" width="11.88671875" style="8" customWidth="1"/>
+    <col min="13" max="13" width="5.5546875" style="8" customWidth="1"/>
+    <col min="14" max="14" width="8.6640625" style="8" customWidth="1"/>
+    <col min="15" max="15" width="5.5546875" style="8" customWidth="1"/>
+    <col min="16" max="16" width="13.5546875" style="8" customWidth="1"/>
     <col min="17" max="17" width="3" style="2" customWidth="1"/>
-    <col min="18" max="18" width="4.140625" style="2" customWidth="1"/>
+    <col min="18" max="18" width="4.109375" style="2" customWidth="1"/>
     <col min="19" max="19" width="3" style="142" customWidth="1"/>
-    <col min="20" max="29" width="10.85546875" style="142" customWidth="1"/>
-    <col min="30" max="30" width="11.42578125" style="187"/>
-    <col min="31" max="34" width="11.42578125" style="167"/>
-    <col min="35" max="35" width="11.42578125" style="7"/>
-    <col min="36" max="16384" width="11.42578125" style="8"/>
+    <col min="20" max="29" width="10.88671875" style="142" customWidth="1"/>
+    <col min="30" max="30" width="11.44140625" style="187"/>
+    <col min="31" max="34" width="11.44140625" style="167"/>
+    <col min="35" max="35" width="11.44140625" style="7"/>
+    <col min="36" max="16384" width="11.44140625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:183" s="4" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:183" s="4" customFormat="1" ht="10.8" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="78"/>
       <c r="B1" s="78"/>
       <c r="C1" s="78"/>
@@ -10530,7 +10530,7 @@
       <c r="AH4" s="135"/>
       <c r="AI4" s="3"/>
     </row>
-    <row r="5" spans="1:183" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:183" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="78"/>
       <c r="B5" s="102" t="s">
         <v>4</v>
@@ -10573,7 +10573,7 @@
       <c r="AH5" s="135"/>
       <c r="AI5" s="3"/>
     </row>
-    <row r="6" spans="1:183" s="5" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:183" s="5" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="72"/>
       <c r="B6" s="106"/>
       <c r="C6" s="72"/>
@@ -11089,7 +11089,7 @@
       <c r="AG12" s="135"/>
       <c r="AH12" s="159"/>
     </row>
-    <row r="13" spans="1:183" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:183" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="82"/>
       <c r="B13" s="78"/>
       <c r="C13" s="268" t="s">
@@ -13509,25 +13509,25 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:GA76"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="10.199999999999999" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4" style="9" customWidth="1"/>
-    <col min="2" max="2" width="3.42578125" style="9" customWidth="1"/>
+    <col min="2" max="2" width="3.44140625" style="9" customWidth="1"/>
     <col min="3" max="3" width="7" style="8" customWidth="1"/>
-    <col min="4" max="4" width="1.42578125" style="8" customWidth="1"/>
+    <col min="4" max="4" width="1.44140625" style="8" customWidth="1"/>
     <col min="5" max="8" width="9" style="8" customWidth="1"/>
-    <col min="9" max="16" width="5.5703125" style="8" customWidth="1"/>
+    <col min="9" max="16" width="5.5546875" style="8" customWidth="1"/>
     <col min="17" max="17" width="3" style="2" customWidth="1"/>
-    <col min="18" max="18" width="4.140625" style="2" customWidth="1"/>
+    <col min="18" max="18" width="4.109375" style="2" customWidth="1"/>
     <col min="19" max="19" width="3" style="142" customWidth="1"/>
-    <col min="20" max="29" width="10.85546875" style="142" customWidth="1"/>
-    <col min="30" max="30" width="11.42578125" style="187"/>
-    <col min="31" max="34" width="11.42578125" style="167"/>
-    <col min="35" max="35" width="11.42578125" style="7"/>
-    <col min="36" max="16384" width="11.42578125" style="8"/>
+    <col min="20" max="29" width="10.88671875" style="142" customWidth="1"/>
+    <col min="30" max="30" width="11.44140625" style="187"/>
+    <col min="31" max="34" width="11.44140625" style="167"/>
+    <col min="35" max="35" width="11.44140625" style="7"/>
+    <col min="36" max="16384" width="11.44140625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:183" s="4" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:183" s="4" customFormat="1" ht="10.8" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="78"/>
       <c r="B1" s="78"/>
       <c r="C1" s="78"/>
@@ -13715,7 +13715,7 @@
       <c r="AH4" s="135"/>
       <c r="AI4" s="3"/>
     </row>
-    <row r="5" spans="1:183" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:183" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="78"/>
       <c r="B5" s="102" t="s">
         <v>4</v>
@@ -13758,7 +13758,7 @@
       <c r="AH5" s="135"/>
       <c r="AI5" s="3"/>
     </row>
-    <row r="6" spans="1:183" s="5" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:183" s="5" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="72"/>
       <c r="B6" s="106"/>
       <c r="C6" s="72"/>
@@ -14274,7 +14274,7 @@
       <c r="AG12" s="135"/>
       <c r="AH12" s="159"/>
     </row>
-    <row r="13" spans="1:183" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:183" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="82"/>
       <c r="B13" s="78"/>
       <c r="C13" s="268" t="s">

</xml_diff>